<commit_message>
feat(F-NAR-008): 24 ATOM de plus (vague 2 partielle)
Histoires, pas des listes. Audio lent déjà recuit pour Raphaël gouttière / flaque.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.POL.001-11.xlsx
+++ b/stories/arbres/ATOM-COL.POL.001-11.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Les poires de Chouchou</t>
+          <t>Le ballon rouge de Chouchou</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Chouchou veut une poire ronde au marché. Il attend, puis il dit bonjour, s'il te plaît, merci. Le filet penche sur le chemin du retour.</t>
+          <t>Chouchou veut le ballon rouge qui tire sur sa ficelle. Il dit bonjour, s'il te plaît, merci. Le ballon tape le lampion jusqu'à la fenêtre.</t>
         </is>
       </c>
     </row>
@@ -1189,12 +1189,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Les sacs en toile pendent à un clou. Ils sentent encore la pluie d'hier. Une goutte tombe du rebord. Elle fait un petit rond dans la flaque. Sur la place, les cagettes claquent. Une pêche roule, puis s'arrête. Ça sent la menthe, près des herbes. En ce moment, Chouchou marche avec maman. Le filet vide tape contre sa jambe. Tu as entendu les cagettes ? Oui, maman. Ça claque. On va voir les poires. Chouchou lève le nez. Ça sent les pommes aussi. Une dame range des poires jaunes. Une autre personne est déjà là. On attend un petit moment. On attend, puis on parle. Chouchou se tient près de maman. La dame se tourne vers eux. On dit bonjour ? Bonjour. Bonjour. La dame incline la tête. Chouchou regarde une poire bien ronde. Elle a des petites taches dorées. Celle-là, maman. Tu la demandes ? Une poire, s'il te plaît. La dame prend la poire. Elle la pose dans le filet. Le filet penche un peu. Merci. Merci. Bravo, Chouchou. Tu as dit bonjour. Tu as dit s'il te plaît. Tu as dit merci. Chouchou tient le filet des deux mains. La poire roule un peu dedans. Elle est fraîche. Oui. Fraîche et lourde. On reprend les trois mots ? Bonjour. S'il te plaît. Merci. C'est ça. Les trois mots. Tu as fait du bon travail. Ils marchent entre les stands. Le filet tape, tout doux.</t>
+          <t>Un lampion rouge se balance sous la corde. La corde va d'un platane à l'autre. La poussière de la place sent encore la pluie. Les dalles sont froides, un peu brillantes. Un accordéon joue tout bas, derrière un stand. Une ficelle danse au-dessus d'une caisse. Le ballon au bout est rouge, tout tendu. Tu as vu la ficelle, Chouchou ? Elle tire. Le ballon veut partir. Il est bien rouge. Je le veux. Celui qui danse. Le vent soulève un peu de papier. Ça sent le sucre filé, tout près. Une miette colle au bord d'une table. On essuie tes mains, d'abord. Voilà. En ce moment, Chouchou tient le panier de maman. Le panier est léger, encore vide. Ils s'arrêtent devant la caisse. Le monsieur du stand parle encore. Il range des ficelles bleues. On attend un petit moment. Il a les mains prises. Le rouge, maman. Il tape la caisse. Oui. Celui-là. Le lampion penche au-dessus d'eux. Une ombre ronde passe sur le nez de Chouchou. Le monsieur pose la dernière ficelle. Il se tourne. Tu demandes, Chouchou. La ficelle rouge tremble encore.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Lise entre à l'étal avec maman. Ça sent les pommes. Lise dit &lt;emphasis level="moderate"&gt;bonjour&lt;/emphasis&gt;. Elle dit s'il te plaît pour une poire. Elle dit merci. Maman sourit. Lise répète : bonjour, s'il te plaît, merci. Elles marchent. Lise tient le filet.&lt;/prosody&gt;&lt;break time="400ms"/&gt;&lt;/speak&gt;</t>
+          <t>Un lampion rouge se balance sous la corde. La corde va d'un platane à l'autre. La poussière de la place sent encore la pluie. Les dalles sont froides, un peu brillantes. Un accordéon joue tout bas, derrière un stand. Une ficelle danse au-dessus d'une caisse. Le ballon au bout est rouge, tout tendu. Tu as vu la ficelle, Chouchou ? Elle tire. Le ballon veut partir. Il est bien rouge. Je le veux. Celui qui danse. Le vent soulève un peu de papier. Ça sent le sucre filé, tout près. Une miette colle au bord d'une table. On essuie tes mains, d'abord. Voilà. En ce moment, Chouchou tient le panier de maman. Le panier est léger, encore vide. Ils s'arrêtent devant la caisse. Le monsieur du stand parle encore. Il range des ficelles bleues. On attend un petit moment. Il a les mains prises. Le rouge, maman. Il tape la caisse. Oui. Celui-là. Le lampion penche au-dessus d'eux. Une ombre ronde passe sur le nez de Chouchou. Le monsieur pose la dernière ficelle. Il se tourne. Tu demandes, Chouchou. La ficelle rouge tremble encore.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1257,7 +1257,7 @@
         <v>0.96</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.12</v>
+        <v>1.22</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1329,59 +1329,46 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Les sacs en toile pendent à un clou.
-narrateur|Ils sentent encore la pluie d'hier.
-narrateur|Une goutte tombe du rebord.
-narrateur|Elle fait un petit rond dans la flaque.
-narrateur|Sur la place, les cagettes claquent.
-narrateur|Une pêche roule, puis s'arrête.
-narrateur|Ça sent la menthe, près des herbes.
-narrateur|En ce moment, Chouchou marche avec maman.
-narrateur|Le filet vide tape contre sa jambe.
-maman|Tu as entendu les cagettes ?
-enfant-m|Oui, maman. Ça claque.
-maman|On va voir les poires.
-narrateur|Chouchou lève le nez.
-narrateur|Ça sent les pommes aussi.
-narrateur|Une dame range des poires jaunes.
-narrateur|Une autre personne est déjà là.
+          <t>narrateur|Un lampion rouge se balance sous la corde.
+narrateur|La corde va d'un platane à l'autre.
+narrateur|La poussière de la place sent encore la pluie.
+narrateur|Les dalles sont froides, un peu brillantes.
+narrateur|Un accordéon joue tout bas, derrière un stand.
+narrateur|Une ficelle danse au-dessus d'une caisse.
+narrateur|Le ballon au bout est rouge, tout tendu.
+maman|Tu as vu la ficelle, Chouchou ?
+enfant-m|Elle tire.
+enfant-m|Le ballon veut partir.
+maman|Il est bien rouge.
+enfant-m|Je le veux.
+enfant-m|Celui qui danse.
+narrateur|Le vent soulève un peu de papier.
+narrateur|Ça sent le sucre filé, tout près.
+narrateur|Une miette colle au bord d'une table.
+maman|On essuie tes mains, d'abord.
+maman|Voilà.
+narrateur|En ce moment, Chouchou tient le panier de maman.
+narrateur|Le panier est léger, encore vide.
+narrateur|Ils s'arrêtent devant la caisse.
+narrateur|Le monsieur du stand parle encore.
+narrateur|Il range des ficelles bleues.
 maman|On attend un petit moment.
-maman|On attend, puis on parle.
-narrateur|Chouchou se tient près de maman.
-narrateur|La dame se tourne vers eux.
-maman|On dit bonjour ?
-enfant-m|Bonjour.
-maman|Bonjour.
-narrateur|La dame incline la tête.
-narrateur|Chouchou regarde une poire bien ronde.
-narrateur|Elle a des petites taches dorées.
-enfant-m|Celle-là, maman.
-maman|Tu la demandes ?
-enfant-m|Une poire, s'il te plaît.
-narrateur|La dame prend la poire.
-narrateur|Elle la pose dans le filet.
-narrateur|Le filet penche un peu.
-enfant-m|Merci.
-maman|Merci.
-maman|Bravo, Chouchou.
-maman|Tu as dit bonjour.
-maman|Tu as dit s'il te plaît.
-maman|Tu as dit merci.
-narrateur|Chouchou tient le filet des deux mains.
-narrateur|La poire roule un peu dedans.
-enfant-m|Elle est fraîche.
-maman|Oui. Fraîche et lourde.
-maman|On reprend les trois mots ?
-enfant-m|Bonjour. S'il te plaît. Merci.
-maman|C'est ça. Les trois mots.
-maman|Tu as fait du bon travail.
-narrateur|Ils marchent entre les stands.
-narrateur|Le filet tape, tout doux.</t>
+maman|Il a les mains prises.
+enfant-m|Le rouge, maman.
+enfant-m|Il tape la caisse.
+maman|Oui.
+maman|Celui-là.
+narrateur|Le lampion penche au-dessus d'eux.
+narrateur|Une ombre ronde passe sur le nez de Chouchou.
+narrateur|Le monsieur pose la dernière ficelle.
+narrateur|Il se tourne.
+maman|Tu demandes, Chouchou.
+narrateur|La ficelle rouge tremble encore.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>goutte,cagettes,marche</t>
+          <t>marche,corde</t>
         </is>
       </c>
     </row>
@@ -1408,12 +1395,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Chouchou parle à la dame. Quels mots dit-il ?</t>
+          <t>Chouchou veut le ballon. Que dit-il ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Lise salue. Quels mots dit-elle ?&lt;/prosody&gt;&lt;break time="250ms"/&gt;&lt;/speak&gt;</t>
+          <t>Chouchou veut le ballon. Que dit-il ?</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -1423,12 +1410,12 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>bonjour</t>
+          <t>s'il te plaît</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>bonjour | s'il te plaît | merci</t>
+          <t>s'il te plaît | merci | bonjour | s'il te plait</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1443,7 +1430,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Trois mots. Bonjour, et ensuite ?</t>
+          <t>Il dit s'il te plaît. Que dit Chouchou ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1564,11 +1551,10 @@
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Chouchou parle à la dame.
-narrateur|Quels mots dit-il ?</t>
-        </is>
-      </c>
-      <c r="AX3" t="inlineStr"/>
+          <t>narrateur|Chouchou veut le ballon.
+narrateur|Que dit-il ?</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1593,12 +1579,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Chouchou a dit bonjour. Il a dit s'il te plaît. Il a dit merci. Tu as dit les trois mots. Bravo. Bonjour. S'il te plaît. Merci. Oui. Même au marché. La poire reste dans le filet. Elle sent un peu le sucré. Tu as fini de tenir le filet ? Oui, maman.</t>
+          <t>Bonjour. Bonjour. Le ballon rouge, s'il te plaît. Celui qui tire. Le monsieur détache la ficelle. Le ballon monte un peu, puis s'arrête. Chouchou tient le bout, des deux mains. Merci. Merci. Le rouge tape le lampion, tout doux. Ça fait un petit bruit de papier. Il est à toi, maintenant. Il est chaud du soleil. Un peu, oui. Plus loin, un moulinet de papier attend. Il est jaune, avec une tige de bois. Il tourne dès qu'on souffle. Tu en veux un, aussi ? Oui. La dame du stand écoute. Bonjour. Le moulinet jaune, s'il te plaît. La dame pose la tige dans sa main. Merci. Tu as demandé, tout clair. Bravo, Chouchou. Le moulinet tourne contre le ballon. Le jaune chatouille le rouge.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Lise a dit &lt;emphasis level="moderate"&gt;bonjour&lt;/emphasis&gt;, s'il te plaît, merci.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Bonjour. Bonjour. Le ballon rouge, s'il te plaît. Celui qui tire. Le monsieur détache la ficelle. Le ballon monte un peu, puis s'arrête. Chouchou tient le bout, des deux mains. Merci. Merci. Le rouge tape le lampion, tout doux. Ça fait un petit bruit de papier. Il est à toi, maintenant. Il est chaud du soleil. Un peu, oui. Plus loin, un moulinet de papier attend. Il est jaune, avec une tige de bois. Il tourne dès qu'on souffle. Tu en veux un, aussi ? Oui. La dame du stand écoute. Bonjour. Le moulinet jaune, s'il te plaît. La dame pose la tige dans sa main. Merci. Tu as demandé, tout clair. Bravo, Chouchou. Le moulinet tourne contre le ballon. Le jaune chatouille le rouge.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1661,7 +1647,7 @@
         <v>0.96</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.22</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1737,20 +1723,41 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Chouchou a dit bonjour.
-narrateur|Il a dit s'il te plaît.
-narrateur|Il a dit merci.
-maman|Tu as dit les trois mots.
-maman|Bravo.
-enfant-m|Bonjour. S'il te plaît. Merci.
-maman|Oui. Même au marché.
-narrateur|La poire reste dans le filet.
-narrateur|Elle sent un peu le sucré.
-maman|Tu as fini de tenir le filet ?
-enfant-m|Oui, maman.</t>
-        </is>
-      </c>
-      <c r="AX4" t="inlineStr"/>
+          <t>enfant-m|Bonjour.
+maman|Bonjour.
+enfant-m|Le ballon rouge, s'il te plaît.
+enfant-m|Celui qui tire.
+narrateur|Le monsieur détache la ficelle.
+narrateur|Le ballon monte un peu, puis s'arrête.
+narrateur|Chouchou tient le bout, des deux mains.
+enfant-m|Merci.
+maman|Merci.
+narrateur|Le rouge tape le lampion, tout doux.
+narrateur|Ça fait un petit bruit de papier.
+maman|Il est à toi, maintenant.
+enfant-m|Il est chaud du soleil.
+maman|Un peu, oui.
+narrateur|Plus loin, un moulinet de papier attend.
+narrateur|Il est jaune, avec une tige de bois.
+narrateur|Il tourne dès qu'on souffle.
+maman|Tu en veux un, aussi ?
+enfant-m|Oui.
+narrateur|La dame du stand écoute.
+enfant-m|Bonjour.
+enfant-m|Le moulinet jaune, s'il te plaît.
+narrateur|La dame pose la tige dans sa main.
+enfant-m|Merci.
+maman|Tu as demandé, tout clair.
+maman|Bravo, Chouchou.
+narrateur|Le moulinet tourne contre le ballon.
+narrateur|Le jaune chatouille le rouge.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>papier</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1775,12 +1782,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Ils quittent la place. Une flaque brille encore. Chouchou saute à côté. Tu tiens bien le filet. La poire est avec moi. Merci, Chouchou. Merci, maman. Le filet tape contre sa jambe. Ça sent encore la menthe, derrière eux. On rentre avec notre poire ? Oui.</t>
+          <t>Ils quittent la place, tout doucement. Le ballon tape chaque lampion, un par un. Il dit bonjour aux lampions. On dirait, oui. Les dalles sèchent sous leurs pas. L'accordéon devient plus loin. À la maison, papa ouvre la fenêtre. C'est un vrai soleil, ça. C'est mon ballon. Tu l'as demandé ? Oui, papa. Bonjour. S'il te plaît. Merci. Et le moulinet ? Il tourne sur le rebord. On le pose près de la vitre. Le ballon touche le bois, tout léger. Le moulinet prend le vent de la rue. Il reste avec nous, ce soir. Oui. Il est rouge.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman range une poire. Lise sourit.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Ils quittent la place, tout doucement. Le ballon tape chaque lampion, un par un. Il dit bonjour aux lampions. On dirait, oui. Les dalles sèchent sous leurs pas. L'accordéon devient plus loin. À la maison, papa ouvre la fenêtre. C'est un vrai soleil, ça. C'est mon ballon. Tu l'as demandé ? Oui, papa. Bonjour. S'il te plaît. Merci. Et le moulinet ? Il tourne sur le rebord. On le pose près de la vitre. Le ballon touche le bois, tout léger. Le moulinet prend le vent de la rue. Il reste avec nous, ce soir. Oui. Il est rouge.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -1843,7 +1850,7 @@
         <v>0.96</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.22</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1911,22 +1918,33 @@
       <c r="AV5" s="2" t="inlineStr"/>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Ils quittent la place.
-narrateur|Une flaque brille encore.
-narrateur|Chouchou saute à côté.
-maman|Tu tiens bien le filet.
-enfant-m|La poire est avec moi.
-maman|Merci, Chouchou.
-enfant-m|Merci, maman.
-narrateur|Le filet tape contre sa jambe.
-narrateur|Ça sent encore la menthe, derrière eux.
-maman|On rentre avec notre poire ?
-enfant-m|Oui.</t>
+          <t>narrateur|Ils quittent la place, tout doucement.
+narrateur|Le ballon tape chaque lampion, un par un.
+enfant-m|Il dit bonjour aux lampions.
+maman|On dirait, oui.
+narrateur|Les dalles sèchent sous leurs pas.
+narrateur|L'accordéon devient plus loin.
+narrateur|À la maison, papa ouvre la fenêtre.
+papa|C'est un vrai soleil, ça.
+enfant-m|C'est mon ballon.
+papa|Tu l'as demandé ?
+enfant-m|Oui, papa.
+enfant-m|Bonjour.
+enfant-m|S'il te plaît.
+enfant-m|Merci.
+papa|Et le moulinet ?
+enfant-m|Il tourne sur le rebord.
+maman|On le pose près de la vitre.
+narrateur|Le ballon touche le bois, tout léger.
+narrateur|Le moulinet prend le vent de la rue.
+papa|Il reste avec nous, ce soir.
+enfant-m|Oui.
+enfant-m|Il est rouge.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>marche</t>
+          <t>pas,fenetre</t>
         </is>
       </c>
     </row>
@@ -1953,12 +1971,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit bonjour. J'ai dit s'il te plaît. J'ai dit merci. Bravo. Tu as fait du bon travail. Le filet est à la maison. L'histoire est finie.</t>
+          <t>Le ballon repose contre la fenêtre. Le lampion de la place n'est plus là. Bonne soirée, Chouchou. Le rouge est rentré. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le ballon repose contre la fenêtre. Le lampion de la place n'est plus là. Bonne soirée, Chouchou. Le rouge est rentré. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -2093,15 +2111,13 @@
       <c r="AV6" s="2" t="inlineStr"/>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai dit bonjour.
-enfant-m|J'ai dit s'il te plaît.
-enfant-m|J'ai dit merci.
-maman|Bravo. Tu as fait du bon travail.
-narrateur|Le filet est à la maison.
+          <t>narrateur|Le ballon repose contre la fenêtre.
+narrateur|Le lampion de la place n'est plus là.
+maman|Bonne soirée, Chouchou.
+papa|Le rouge est rentré.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX6" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:AV6"/>
@@ -2120,7 +2136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2165,6 +2181,13 @@
       <c r="A6" t="inlineStr">
         <is>
           <t>F-NAR-009 ouverture du monde, fusion agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(F-NAR-019): ATOM-COL.POL.001-11 Les poires de Chouchou
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.POL.001-11.xlsx
+++ b/stories/arbres/ATOM-COL.POL.001-11.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le ballon rouge de Chouchou</t>
+          <t>Les poires de Chouchou</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>place du village, lampions, puis fenêtre</t>
+          <t>marché, sacs en toile au clou, pluie d'hier, goutte, rond, filet, poires jaunes, étal</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Chouchou veut le ballon rouge qui tire sur sa ficelle. Il dit bonjour, s'il te plaît, merci. Le ballon tape le lampion jusqu'à la fenêtre.</t>
+          <t>Les sacs en toile pendent à un clou. Ils sentent la pluie d'hier. Une goutte fait un rond. Sur un sac, un éclat de sac brille. Chouchou veut des poires maintenant. Elle avance trop vite : l'éclat glisse, la dame ne se tourne pas. Elle refuse de foncer, dit bonjour. Merci vécu. Une poire trop vite : le filet penche. Elle refuse, demande. Sur la toile, l'éclat de sac tient.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un lampion rouge se balance sous la corde. La corde va d'un platane à l'autre. La poussière de la place sent encore la pluie. Les dalles sont froides, un peu brillantes. Un accordéon joue tout bas, derrière un stand. Une ficelle danse au-dessus d'une caisse. Le ballon au bout est rouge, tout tendu. Tu as vu la ficelle, Chouchou ? Elle tire. Le ballon veut partir. Il est bien rouge. Je le veux. Celui qui danse. Le vent soulève un peu de papier. Ça sent le sucre filé, tout près. Une miette colle au bord d'une table. On essuie tes mains, d'abord. Voilà. En ce moment, Chouchou tient le panier de maman. Le panier est léger, encore vide. Ils s'arrêtent devant la caisse. Le monsieur du stand parle encore. Il range des ficelles bleues. On attend un petit moment. Il a les mains prises. Le rouge, maman. Il tape la caisse. Oui. Celui-là. Le lampion penche au-dessus d'eux. Une ombre ronde passe sur le nez de Chouchou. Le monsieur pose la dernière ficelle. Il se tourne. Tu demandes, Chouchou. La ficelle rouge tremble encore.</t>
+          <t>Un clou tient des sacs en toile, lourds d'eau. Ils sentent la pluie d'hier. Une goutte tombe du rebord. Elle fait un petit rond dans la flaque. Sur un sac, un éclat de sac brille. Il brille, papa ! C'est l'eau, sur la toile ? Oui, tout petit. Chouchou connaît cette place, un peu. Les cagettes claquent sur la pierre. Une pêche roule, puis s'arrête. Tu as entendu les cagettes ? Oui, maman. Ça claque. On va voir les poires ? Les jaunes, maintenant ! Le filet vide tape contre sa jambe. Il est léger. On le remplit, tout à l'heure. Tout de suite ! Ça sent la menthe, près des herbes. Ça sent les pommes aussi. En ce moment, Chouchou marche vers les poires. La dame range des poires jaunes. Elles sont rondes, avec des taches dorées. Celles-là, maman ! Tu les prends, Chouchou ? Oui, maintenant ! Chouchou avance le filet trop vite. Les sacs se balancent au clou. L'éclat de sac glisse sur la toile. Oh. La dame ne se tourne pas. Ses mains restent dans les poires. Oh. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu parles à la dame, Chouchou ? Papa s'accroupit à la même hauteur. Oui, papa. Les mots se perdent près des poires. Personne n'entend la fin. Chouchou referme la bouche, un instant. Le filet reste vide, un peu lourd.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Un lampion rouge se balance sous la corde. La corde va d'un platane à l'autre. La poussière de la place sent encore la pluie. Les dalles sont froides, un peu brillantes. Un accordéon joue tout bas, derrière un stand. Une ficelle danse au-dessus d'une caisse. Le ballon au bout est rouge, tout tendu. Tu as vu la ficelle, Chouchou ? Elle tire. Le ballon veut partir. Il est bien rouge. Je le veux. Celui qui danse. Le vent soulève un peu de papier. Ça sent le sucre filé, tout près. Une miette colle au bord d'une table. On essuie tes mains, d'abord. Voilà. En ce moment, Chouchou tient le panier de maman. Le panier est léger, encore vide. Ils s'arrêtent devant la caisse. Le monsieur du stand parle encore. Il range des ficelles bleues. On attend un petit moment. Il a les mains prises. Le rouge, maman. Il tape la caisse. Oui. Celui-là. Le lampion penche au-dessus d'eux. Une ombre ronde passe sur le nez de Chouchou. Le monsieur pose la dernière ficelle. Il se tourne. Tu demandes, Chouchou. La ficelle rouge tremble encore.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un clou tient des sacs en toile, lourds d'eau. Ils sentent la pluie d'hier. Une goutte tombe du rebord. Elle fait un petit rond dans la flaque. Sur un sac, un &lt;emphasis level="moderate"&gt;éclat de sac&lt;/emphasis&gt; brille. Il brille, papa ! C'est l'eau, sur la toile ? Oui, tout petit. Chouchou connaît cette place, un peu. Les cagettes claquent sur la pierre. Une pêche roule, puis s'arrête. Tu as entendu les cagettes ? Oui, maman. Ça claque. On va voir les poires ? Les jaunes, maintenant ! Le filet vide tape contre sa jambe. Il est léger. On le remplit, tout à l'heure. Tout de suite ! Ça sent la menthe, près des herbes. Ça sent les pommes aussi. En ce moment, Chouchou marche vers les poires. La dame range des poires jaunes. Elles sont rondes, avec des taches dorées. Celles-là, maman ! Tu les prends, Chouchou ? Oui, maintenant ! Chouchou avance le filet trop vite. Les sacs se balancent au clou. L'éclat de sac glisse sur la toile. Oh. La dame ne se tourne pas. Ses mains restent dans les poires. Oh. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu parles à la dame, Chouchou ? Papa s'accroupit à la même hauteur. Oui, papa. Les mots se perdent près des poires. Personne n'entend la fin. Chouchou referme la bouche, un instant. Le filet reste vide, un peu lourd.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Lise entre à l'étal avec maman. Ça sent les pommes. Lise dit &lt;emphasis&gt;bonjour&lt;/emphasis&gt;. Elle dit s'il te plaît pour une poire. Elle dit merci. Maman sourit. Lise répète : bonjour, s'il te plaît, merci. Elles marchent. Lise tient le filet. [pause]</t>
+          <t>Un clou tient des sacs en toile, lourds d'eau. Ils sentent la pluie d'hier. Une goutte tombe du rebord. Elle fait un petit rond dans la flaque. Sur un sac, un &lt;emphasis&gt;éclat de sac&lt;/emphasis&gt; brille. Il brille, papa ! C'est l'eau, sur la toile ? Oui, tout petit. Chouchou connaît cette place, un peu. Les cagettes claquent sur la pierre. Une pêche roule, puis s'arrête. Tu as entendu les cagettes ? Oui, maman. Ça claque. On va voir les poires ? Les jaunes, maintenant ! Le filet vide tape contre sa jambe. Il est léger. On le remplit, tout à l'heure. Tout de suite ! Ça sent la menthe, près des herbes. Ça sent les pommes aussi. En ce moment, Chouchou marche vers les poires. La dame range des poires jaunes. Elles sont rondes, avec des taches dorées. Celles-là, maman ! Tu les prends, Chouchou ? Oui, maintenant ! Chouchou avance le filet trop vite. Les sacs se balancent au clou. L'éclat de sac glisse sur la toile. Oh. La dame ne se tourne pas. Ses mains restent dans les poires. Oh. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu parles à la dame, Chouchou ? Papa s'accroupit à la même hauteur. Oui, papa. Les mots se perdent près des poires. Personne n'entend la fin. Chouchou referme la bouche, un instant. Le filet reste vide, un peu lourd. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>bonjour</t>
+          <t>éclat de sac</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,49 +1326,62 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_les_poires_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un lampion rouge se balance sous la corde.
-narrateur|La corde va d'un platane à l'autre.
-narrateur|La poussière de la place sent encore la pluie.
-narrateur|Les dalles sont froides, un peu brillantes.
-narrateur|Un accordéon joue tout bas, derrière un stand.
-narrateur|Une ficelle danse au-dessus d'une caisse.
-narrateur|Le ballon au bout est rouge, tout tendu.
-maman|Tu as vu la ficelle, Chouchou ?
-enfant-m|Elle tire.
-enfant-m|Le ballon veut partir.
-maman|Il est bien rouge.
-enfant-m|Je le veux.
-enfant-m|Celui qui danse.
-narrateur|Le vent soulève un peu de papier.
-narrateur|Ça sent le sucre filé, tout près.
-narrateur|Une miette colle au bord d'une table.
-maman|On essuie tes mains, d'abord.
-maman|Voilà.
-narrateur|En ce moment, Chouchou tient le panier de maman.
-narrateur|Le panier est léger, encore vide.
-narrateur|Ils s'arrêtent devant la caisse.
-narrateur|Le monsieur du stand parle encore.
-narrateur|Il range des ficelles bleues.
-maman|On attend un petit moment.
-maman|Il a les mains prises.
-enfant-m|Le rouge, maman.
-enfant-m|Il tape la caisse.
-maman|Oui.
-maman|Celui-là.
-narrateur|Le lampion penche au-dessus d'eux.
-narrateur|Une ombre ronde passe sur le nez de Chouchou.
-narrateur|Le monsieur pose la dernière ficelle.
-narrateur|Il se tourne.
-maman|Tu demandes, Chouchou.
-narrateur|La ficelle rouge tremble encore.</t>
+          <t>narrateur|Un clou tient des sacs en toile, lourds d'eau.
+narrateur|Ils sentent la pluie d'hier.
+narrateur|Une goutte tombe du rebord.
+narrateur|Elle fait un petit rond dans la flaque.
+narrateur|Sur un sac, un éclat de sac brille.
+enfant-f|Il brille, papa !
+papa|C'est l'eau, sur la toile ?
+enfant-f|Oui, tout petit.
+narrateur|Chouchou connaît cette place, un peu.
+narrateur|Les cagettes claquent sur la pierre.
+narrateur|Une pêche roule, puis s'arrête.
+maman|Tu as entendu les cagettes ?
+enfant-f|Oui, maman.
+enfant-f|Ça claque.
+papa|On va voir les poires ?
+enfant-f|Les jaunes, maintenant !
+narrateur|Le filet vide tape contre sa jambe.
+enfant-f|Il est léger.
+maman|On le remplit, tout à l'heure.
+enfant-f|Tout de suite !
+narrateur|Ça sent la menthe, près des herbes.
+enfant-f|Ça sent les pommes aussi.
+narrateur|En ce moment, Chouchou marche vers les poires.
+narrateur|La dame range des poires jaunes.
+narrateur|Elles sont rondes, avec des taches dorées.
+enfant-f|Celles-là, maman !
+papa|Tu les prends, Chouchou ?
+enfant-f|Oui, maintenant !
+narrateur|Chouchou avance le filet trop vite.
+narrateur|Les sacs se balancent au clou.
+narrateur|L'éclat de sac glisse sur la toile.
+enfant-f|Oh.
+narrateur|La dame ne se tourne pas.
+narrateur|Ses mains restent dans les poires.
+enfant-f|Oh.
+narrateur|Le sourire de Chouchou disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+papa|Tu parles à la dame, Chouchou ?
+narrateur|Papa s'accroupit à la même hauteur.
+enfant-f|Oui, papa.
+narrateur|Les mots se perdent près des poires.
+narrateur|Personne n'entend la fin.
+narrateur|Chouchou referme la bouche, un instant.
+narrateur|Le filet reste vide, un peu lourd.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>marche,corde</t>
+          <t>goutte,cagettes,marche</t>
         </is>
       </c>
     </row>
@@ -1395,27 +1408,27 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Chouchou veut le ballon. Que dit-il ?</t>
+          <t>Chouchou parle à la dame. Que dit-elle ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Chouchou veut le ballon. Que dit-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Chouchou parle à la &lt;emphasis level="moderate"&gt;dame&lt;/emphasis&gt;. Que dit-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Lise salue. Quels mots dit-elle ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Chouchou parle à la &lt;emphasis&gt;dame&lt;/emphasis&gt;. Que dit-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>s'il te plaît</t>
+          <t>bonjour</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>s'il te plaît | merci | bonjour | s'il te plait</t>
+          <t>bonjour | s'il te plaît | merci | s'il te plait</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1430,7 +1443,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Il dit s'il te plaît. Que dit Chouchou ?</t>
+          <t>Elle dit bonjour. Que dit Chouchou ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1468,18 +1481,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1494,34 +1507,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>dame</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1530,29 +1547,29 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_dit_bonjour_en_parlant_a_la_dame; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Chouchou veut le ballon.
-narrateur|Que dit-il ?</t>
+          <t>narrateur|Chouchou parle à la dame.
+narrateur|Que dit-elle ?</t>
         </is>
       </c>
     </row>
@@ -1579,17 +1596,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. Le ballon rouge, s'il te plaît. Celui qui tire. Le monsieur détache la ficelle. Le ballon monte un peu, puis s'arrête. Chouchou tient le bout, des deux mains. Merci. Merci. Le rouge tape le lampion, tout doux. Ça fait un petit bruit de papier. Il est à toi, maintenant. Il est chaud du soleil. Un peu, oui. Plus loin, un moulinet de papier attend. Il est jaune, avec une tige de bois. Il tourne dès qu'on souffle. Tu en veux un, aussi ? Oui. La dame du stand écoute. Bonjour. Le moulinet jaune, s'il te plaît. La dame pose la tige dans sa main. Merci. Tu as demandé, tout clair. Bravo, Chouchou. Le moulinet tourne contre le ballon. Le jaune chatouille le rouge.</t>
+          <t>Chouchou avance le filet trop vite. Les poires, les jaunes, pour nous ! Les mots se bousculent dans sa bouche. La dame ne prend pas le filet. Oh. Le sourire ne revient pas. Chouchou refuse de foncer. Elle recule le filet, un peu. Le filet est vide, Chouchou ? Papa reste à sa hauteur. La flaque ronde est sous tes pieds. Maman n'a pas fini non plus. Chouchou attend que le silence arrive. Sur la toile, l'éclat de sac brille. Il est là. Bonjour. Bonjour. Des poires, s'il te plaît. Les jaunes, s'il te plaît. La dame pose des poires dans le filet. Le filet penche, un peu. Merci. Merci, Chouchou. Papa a entendu toute la phrase. Tu tiens le filet des deux mains ? Oui, maman. Elles sont fraîches. Tu parles du rond, si tu veux ? La goutte a fait un rond. On rentre, Chouchou ? Oui. Une lumière jaune vient des poires. L'odeur de menthe reste sur la place.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. Le ballon rouge, s'il te plaît. Celui qui tire. Le monsieur détache la ficelle. Le ballon monte un peu, puis s'arrête. Chouchou tient le bout, des deux mains. Merci. Merci. Le rouge tape le lampion, tout doux. Ça fait un petit bruit de papier. Il est à toi, maintenant. Il est chaud du soleil. Un peu, oui. Plus loin, un moulinet de papier attend. Il est jaune, avec une tige de bois. Il tourne dès qu'on souffle. Tu en veux un, aussi ? Oui. La dame du stand écoute. Bonjour. Le moulinet jaune, s'il te plaît. La dame pose la tige dans sa main. Merci. Tu as demandé, tout clair. Bravo, Chouchou. Le moulinet tourne contre le ballon. Le jaune chatouille le rouge.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Chouchou avance le filet trop vite. Les poires, les jaunes, pour nous ! Les mots se bousculent dans sa bouche. La dame ne prend pas le filet. Oh. Le sourire ne revient pas. Chouchou refuse de foncer. Elle recule le filet, un peu. Le filet est vide, Chouchou ? Papa reste à sa hauteur. La flaque ronde est sous tes pieds. Maman n'a pas fini non plus. Chouchou attend que le silence arrive. Sur la toile, l'éclat de sac brille. Il est là. &lt;emphasis level="moderate"&gt;Bonjour&lt;/emphasis&gt;. Bonjour. Des poires, s'il te plaît. Les jaunes, s'il te plaît. La dame pose des poires dans le filet. Le filet penche, un peu. Merci. Merci, Chouchou. Papa a entendu toute la phrase. Tu tiens le filet des deux mains ? Oui, maman. Elles sont fraîches. Tu parles du rond, si tu veux ? La goutte a fait un rond. On rentre, Chouchou ? Oui. Une lumière jaune vient des poires. L'odeur de menthe reste sur la place.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Lise a dit &lt;emphasis&gt;bonjour&lt;/emphasis&gt;, s'il te plaît, merci. [pause]</t>
+          <t>Chouchou avance le filet trop vite. Les poires, les jaunes, pour nous ! Les mots se bousculent dans sa bouche. La dame ne prend pas le filet. Oh. Le sourire ne revient pas. Chouchou refuse de foncer. Elle recule le filet, un peu. Le filet est vide, Chouchou ? Papa reste à sa hauteur. La flaque ronde est sous tes pieds. Maman n'a pas fini non plus. Chouchou attend que le silence arrive. Sur la toile, l'éclat de sac brille. Il est là. &lt;emphasis&gt;Bonjour&lt;/emphasis&gt;. Bonjour. Des poires, s'il te plaît. Les jaunes, s'il te plaît. La dame pose des poires dans le filet. Le filet penche, un peu. Merci. Merci, Chouchou. Papa a entendu toute la phrase. Tu tiens le filet des deux mains ? Oui, maman. Elles sont fraîches. Tu parles du rond, si tu veux ? La goutte a fait un rond. On rentre, Chouchou ? Oui. Une lumière jaune vient des poires. L'odeur de menthe reste sur la place. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1636,7 +1653,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1644,10 +1661,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1670,30 +1687,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>bonjour</t>
+          <t>Bonjour</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1702,10 +1719,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1718,44 +1735,49 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_attend_puis_dit_bonjour; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>enfant-m|Bonjour.
-maman|Bonjour.
-enfant-m|Le ballon rouge, s'il te plaît.
-enfant-m|Celui qui tire.
-narrateur|Le monsieur détache la ficelle.
-narrateur|Le ballon monte un peu, puis s'arrête.
-narrateur|Chouchou tient le bout, des deux mains.
-enfant-m|Merci.
-maman|Merci.
-narrateur|Le rouge tape le lampion, tout doux.
-narrateur|Ça fait un petit bruit de papier.
-maman|Il est à toi, maintenant.
-enfant-m|Il est chaud du soleil.
-maman|Un peu, oui.
-narrateur|Plus loin, un moulinet de papier attend.
-narrateur|Il est jaune, avec une tige de bois.
-narrateur|Il tourne dès qu'on souffle.
-maman|Tu en veux un, aussi ?
-enfant-m|Oui.
-narrateur|La dame du stand écoute.
-enfant-m|Bonjour.
-enfant-m|Le moulinet jaune, s'il te plaît.
-narrateur|La dame pose la tige dans sa main.
-enfant-m|Merci.
-maman|Tu as demandé, tout clair.
-maman|Bravo, Chouchou.
-narrateur|Le moulinet tourne contre le ballon.
-narrateur|Le jaune chatouille le rouge.</t>
+          <t>narrateur|Chouchou avance le filet trop vite.
+enfant-f|Les poires, les jaunes, pour nous !
+narrateur|Les mots se bousculent dans sa bouche.
+narrateur|La dame ne prend pas le filet.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Chouchou refuse de foncer.
+narrateur|Elle recule le filet, un peu.
+papa|Le filet est vide, Chouchou ?
+narrateur|Papa reste à sa hauteur.
+maman|La flaque ronde est sous tes pieds.
+narrateur|Maman n'a pas fini non plus.
+narrateur|Chouchou attend que le silence arrive.
+narrateur|Sur la toile, l'éclat de sac brille.
+enfant-f|Il est là.
+enfant-f|Bonjour.
+papa|Bonjour.
+enfant-f|Des poires, s'il te plaît.
+enfant-f|Les jaunes, s'il te plaît.
+narrateur|La dame pose des poires dans le filet.
+narrateur|Le filet penche, un peu.
+enfant-f|Merci.
+papa|Merci, Chouchou.
+narrateur|Papa a entendu toute la phrase.
+maman|Tu tiens le filet des deux mains ?
+enfant-f|Oui, maman.
+enfant-f|Elles sont fraîches.
+papa|Tu parles du rond, si tu veux ?
+enfant-f|La goutte a fait un rond.
+maman|On rentre, Chouchou ?
+enfant-f|Oui.
+narrateur|Une lumière jaune vient des poires.
+narrateur|L'odeur de menthe reste sur la place.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>papier</t>
+          <t>marche,filet</t>
         </is>
       </c>
     </row>
@@ -1782,17 +1804,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Ils quittent la place, tout doucement. Le ballon tape chaque lampion, un par un. Il dit bonjour aux lampions. On dirait, oui. Les dalles sèchent sous leurs pas. L'accordéon devient plus loin. À la maison, papa ouvre la fenêtre. C'est un vrai soleil, ça. C'est mon ballon. Tu l'as demandé ? Oui, papa. Bonjour. S'il te plaît. Merci. Et le moulinet ? Il tourne sur le rebord. On le pose près de la vitre. Le ballon touche le bois, tout léger. Le moulinet prend le vent de la rue. Il reste avec nous, ce soir. Oui. Il est rouge.</t>
+          <t>Chouchou quitte la place avec papa et maman. Une flaque brille, ronde, près de la pierre. La menthe reste dans l'air. Le filet est lourd, papa. Les poires sont dedans, oui. À la maison, la table sent les poires. Je prends une poire, maintenant ! Chouchou avance la main trop vite. Une poire roule vers le bord du filet. Oh. Papa n'a pas fini sa phrase. Le filet penche, Chouchou. Les deux voix se mélangent. Oh. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Elle écoute la cuisine, un instant. Elle pose la main, sans presser. S'il te plaît, une poire ? Oui, une petite. Elle est fraîche, maman. Tu restes un peu ? Oui, papa. Le filet est près de l'évier. On le pose ? Oui, sur le bois. La poire sent le sucré. Elle colle aux doigts. Comme la toile, oui.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Ils quittent la place, tout doucement. Le ballon tape chaque lampion, un par un. Il dit bonjour aux lampions. On dirait, oui. Les dalles sèchent sous leurs pas. L'accordéon devient plus loin. À la maison, papa ouvre la fenêtre. C'est un vrai soleil, ça. C'est mon ballon. Tu l'as demandé ? Oui, papa. Bonjour. S'il te plaît. Merci. Et le moulinet ? Il tourne sur le rebord. On le pose près de la vitre. Le ballon touche le bois, tout léger. Le moulinet prend le vent de la rue. Il reste avec nous, ce soir. Oui. Il est rouge.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Chouchou quitte la place avec papa et maman. Une flaque brille, ronde, près de la pierre. La menthe reste dans l'air. Le &lt;emphasis level="moderate"&gt;filet&lt;/emphasis&gt; est lourd, papa. Les poires sont dedans, oui. À la maison, la table sent les poires. Je prends une poire, maintenant ! Chouchou avance la main trop vite. Une poire roule vers le bord du filet. Oh. Papa n'a pas fini sa phrase. Le filet penche, Chouchou. Les deux voix se mélangent. Oh. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Elle écoute la cuisine, un instant. Elle pose la main, sans presser. S'il te plaît, une poire ? Oui, une petite. Elle est fraîche, maman. Tu restes un peu ? Oui, papa. Le filet est près de l'évier. On le pose ? Oui, sur le bois. La poire sent le sucré. Elle colle aux doigts. Comme la toile, oui.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman range une poire. Lise sourit. [pause]</t>
+          <t>Chouchou quitte la place avec papa et maman. Une flaque brille, ronde, près de la pierre. La menthe reste dans l'air. Le &lt;emphasis&gt;filet&lt;/emphasis&gt; est lourd, papa. Les poires sont dedans, oui. À la maison, la table sent les poires. Je prends une poire, maintenant ! Chouchou avance la main trop vite. Une poire roule vers le bord du filet. Oh. Papa n'a pas fini sa phrase. Le filet penche, Chouchou. Les deux voix se mélangent. Oh. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Elle écoute la cuisine, un instant. Elle pose la main, sans presser. S'il te plaît, une poire ? Oui, une petite. Elle est fraîche, maman. Tu restes un peu ? Oui, papa. Le filet est près de l'évier. On le pose ? Oui, sur le bois. La poire sent le sucré. Elle colle aux doigts. Comme la toile, oui. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1839,7 +1861,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1847,10 +1869,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1871,28 +1893,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>filet</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1901,10 +1927,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1915,36 +1941,47 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_sur_la_poire; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Ils quittent la place, tout doucement.
-narrateur|Le ballon tape chaque lampion, un par un.
-enfant-m|Il dit bonjour aux lampions.
-maman|On dirait, oui.
-narrateur|Les dalles sèchent sous leurs pas.
-narrateur|L'accordéon devient plus loin.
-narrateur|À la maison, papa ouvre la fenêtre.
-papa|C'est un vrai soleil, ça.
-enfant-m|C'est mon ballon.
-papa|Tu l'as demandé ?
-enfant-m|Oui, papa.
-enfant-m|Bonjour.
-enfant-m|S'il te plaît.
-enfant-m|Merci.
-papa|Et le moulinet ?
-enfant-m|Il tourne sur le rebord.
-maman|On le pose près de la vitre.
-narrateur|Le ballon touche le bois, tout léger.
-narrateur|Le moulinet prend le vent de la rue.
-papa|Il reste avec nous, ce soir.
-enfant-m|Oui.
-enfant-m|Il est rouge.</t>
+          <t>narrateur|Chouchou quitte la place avec papa et maman.
+narrateur|Une flaque brille, ronde, près de la pierre.
+narrateur|La menthe reste dans l'air.
+enfant-f|Le filet est lourd, papa.
+papa|Les poires sont dedans, oui.
+narrateur|À la maison, la table sent les poires.
+enfant-f|Je prends une poire, maintenant !
+narrateur|Chouchou avance la main trop vite.
+narrateur|Une poire roule vers le bord du filet.
+enfant-f|Oh.
+narrateur|Papa n'a pas fini sa phrase.
+papa|Le filet penche, Chouchou.
+narrateur|Les deux voix se mélangent.
+enfant-f|Oh.
+narrateur|Chouchou refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Elle écoute la cuisine, un instant.
+narrateur|Elle pose la main, sans presser.
+enfant-f|S'il te plaît, une poire ?
+maman|Oui, une petite.
+enfant-f|Elle est fraîche, maman.
+papa|Tu restes un peu ?
+enfant-f|Oui, papa.
+maman|Le filet est près de l'évier.
+enfant-f|On le pose ?
+papa|Oui, sur le bois.
+narrateur|La poire sent le sucré.
+enfant-f|Elle colle aux doigts.
+maman|Comme la toile, oui.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>pas,fenetre</t>
+          <t>marche,table</t>
         </is>
       </c>
     </row>
@@ -1971,17 +2008,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le ballon repose contre la fenêtre. Le lampion de la place n'est plus là. Bonne soirée, Chouchou. Le rouge est rentré.</t>
+          <t>Ils restent près de la table. Maman accroche le sac en toile au clou. Comme au marché, papa. Tu le vois, toi ? Oui, sur la toile. On est bien, ici. Chouchou glisse le doigt, sans se presser. On le sent, maman. Tu le sens sur tes doigts ? Oui, il colle. Le filet est rentré lourd. Oui, avec les poires. L'odeur de menthe reste dans la cuisine. Il est là, maman. Oui, sur la toile. L'éclat de sac tient sur la toile.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le ballon repose contre la fenêtre. Le lampion de la place n'est plus là. Bonne soirée, Chouchou. Le rouge est rentré.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la table. Maman accroche le sac en toile au clou. Comme au marché, papa. Tu le vois, toi ? Oui, sur la toile. On est bien, ici. Chouchou glisse le doigt, sans se presser. On le sent, maman. Tu le sens sur tes doigts ? Oui, il colle. Le filet est rentré lourd. Oui, avec les poires. L'odeur de menthe reste dans la cuisine. Il est là, maman. Oui, sur la toile. L'&lt;emphasis level="moderate"&gt;éclat de sac&lt;/emphasis&gt; tient sur la toile.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la table. Maman accroche le sac en toile au clou. Comme au marché, papa. Tu le vois, toi ? Oui, sur la toile. On est bien, ici. Chouchou glisse le doigt, sans se presser. On le sent, maman. Tu le sens sur tes doigts ? Oui, il colle. Le filet est rentré lourd. Oui, avec les poires. L'odeur de menthe reste dans la cuisine. Il est là, maman. Oui, sur la toile. L'&lt;emphasis&gt;éclat de sac&lt;/emphasis&gt; tient sur la toile.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2028,18 +2065,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2048,12 +2085,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2062,17 +2099,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de sac</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2081,11 +2122,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2094,27 +2135,48 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_la_toile; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le ballon repose contre la fenêtre.
-narrateur|Le lampion de la place n'est plus là.
-maman|Bonne soirée, Chouchou.
-papa|Le rouge est rentré.</t>
+          <t>narrateur|Ils restent près de la table.
+narrateur|Maman accroche le sac en toile au clou.
+enfant-f|Comme au marché, papa.
+papa|Tu le vois, toi ?
+enfant-f|Oui, sur la toile.
+maman|On est bien, ici.
+narrateur|Chouchou glisse le doigt, sans se presser.
+enfant-f|On le sent, maman.
+maman|Tu le sens sur tes doigts ?
+enfant-f|Oui, il colle.
+papa|Le filet est rentré lourd.
+enfant-f|Oui, avec les poires.
+narrateur|L'odeur de menthe reste dans la cuisine.
+enfant-f|Il est là, maman.
+maman|Oui, sur la toile.
+narrateur|L'éclat de sac tient sur la toile.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>sac,cuisine</t>
         </is>
       </c>
     </row>
@@ -2135,7 +2197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2192,6 +2254,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>